<commit_message>
Real KES term dates, cut prose to bullets
Pulled KES's own term dates PDF directly from kesbath.com rather than
guessing:
- Autumn half term is 17 to 30 October 2026, two weeks, not the one
  week previously assumed. Both Wk5 (20 Oct) and Wk6 (27 Oct) fall
  inside it, not just Wk6.
- Autumn term ends Wed 16 Dec 2026, spring term starts Wed 6 Jan 2027.
  Wk14 (22 Dec), Wk15 (29 Dec) and Wk16 (5 Jan), three sessions not
  two, are outside term time.

Every block (School Calendar, Today, Daily Practice, Mock Paper) is
now bullet points, explanatory sentences cut.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WGnPYmvuvjhBfpkVc2KCDJ
</commit_message>
<xml_diff>
--- a/resources/Maths-Topics-PDFs.xlsx
+++ b/resources/Maths-Topics-PDFs.xlsx
@@ -73,6 +73,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FBE7E4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FDF0D5"/>
       </patternFill>
     </fill>
@@ -84,11 +89,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E6EEE0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FBE7E4"/>
       </patternFill>
     </fill>
     <fill>
@@ -149,15 +149,15 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -185,6 +185,33 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -194,22 +221,13 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -218,25 +236,7 @@
     <xf numFmtId="165" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -622,7 +622,7 @@
     <col width="34" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="52" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -635,328 +635,303 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>For King Edward's School, Bath. Exam Sat 16 Jan 2027, confirmed on kesbath.com. Application deadline Mon 16 Nov 2026.</t>
+          <t>King Edward's School, Bath. Exam Sat 16 Jan 2027. Application deadline Mon 16 Nov 2026.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>First session tonight, Tue 22 Sep. Weekly Tuesdays after that. Every link below was working as of 22 Sep 2026.</t>
+          <t>First session tonight, Tue 22 Sep. Weekly Tuesdays after that.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>TODAY, first session: see where she is at</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="26" customHeight="1">
+          <t>SCHOOL CALENDAR (KES own term dates PDF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Before starting Addition and Subtraction below, spend the first 15 to 20 minutes on an informal look across all four operations, not a test, no marks, just watching what she does.</t>
+          <t>• Autumn half term: 17 to 30 October 2026, two weeks. Wk5 (20 Oct) and Wk6 (27 Oct) below both fall inside it.</t>
         </is>
       </c>
       <c r="B6" s="5" t="n"/>
       <c r="C6" s="5" t="n"/>
       <c r="D6" s="5" t="n"/>
     </row>
-    <row r="7" ht="26" customHeight="1">
+    <row r="7" ht="20" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Give her two or three questions each from the Addition, Subtraction, Multiplication and Division worksheets in the table below, plus a quick look at one Fraction of Amounts and one Percentages of Amounts question, to see the upper end too.</t>
+          <t>• Autumn term ends: Wed 16 Dec 2026. Wk13 (15 Dec) is fine, still term time.</t>
         </is>
       </c>
       <c r="B7" s="5" t="n"/>
       <c r="C7" s="5" t="n"/>
       <c r="D7" s="5" t="n"/>
     </row>
-    <row r="8" ht="26" customHeight="1">
+    <row r="8" ht="20" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Watch for: which operation she reaches for confidently, where she hesitates or guesses, whether she works in her head or writes it down, and whether she can explain how she got an answer.</t>
+          <t>• Spring term starts: Wed 6 Jan 2027. Wk14 (22 Dec), Wk15 (29 Dec) and Wk16 (5 Jan) are all school holiday, not term time.</t>
         </is>
       </c>
       <c r="B8" s="5" t="n"/>
       <c r="C8" s="5" t="n"/>
       <c r="D8" s="5" t="n"/>
     </row>
-    <row r="9" ht="26" customHeight="1">
+    <row r="9" ht="20" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Use what you see to decide how the rest of tonight goes. If all four operations are already solid, move faster into next week's content instead of spending the full session on Addition and Subtraction.</t>
+          <t>• Decide: keep these five sessions as holiday tutoring, or move them and shift the rest of the schedule.</t>
         </is>
       </c>
       <c r="B9" s="5" t="n"/>
       <c r="C9" s="5" t="n"/>
       <c r="D9" s="5" t="n"/>
     </row>
-    <row r="10" ht="26" customHeight="1">
+    <row r="10" ht="20" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>No score needed, a one line note afterwards on what was solid and what was not is enough to plan the next few weeks around.</t>
+          <t>KES term dates 2026-27, PDF</t>
         </is>
       </c>
       <c r="B10" s="5" t="n"/>
       <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>DAILY PRACTICE (separate from the weekly topic session below)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="26" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Most days, about 10 to 15 minutes, not a new topic, just keeping everything moving. This is Corbettmaths Primary 5-a-day.</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-    </row>
-    <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Start on the Silver tier. Move to Gold if Silver is too easy after a week or two, or down to Bronze if it is a struggle.</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
-    </row>
-    <row r="15" ht="26" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Each tier has one PDF per month, five questions a day down the page. Print once a month, not once a day.</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="n"/>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="7" t="n"/>
-    </row>
-    <row r="16" ht="26" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Answers are on a separate page for each month, linked below, since the site does not keep one fixed answers file per month.</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="n"/>
-      <c r="C16" s="7" t="n"/>
-      <c r="D16" s="7" t="n"/>
-    </row>
-    <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>Add 2 to 3 minutes of times tables recall before or after the 5-a-day, self tested, no worksheet needed.</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="n"/>
-      <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="n"/>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>5-a-day home page, start here, always current</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="n"/>
-      <c r="C18" s="7" t="n"/>
-      <c r="D18" s="8" t="inlineStr">
+          <t>TODAY: see where she is at, before Addition and Subtraction below</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>• 15 to 20 min, no marks: 2 to 3 questions each from Addition, Subtraction, Multiplication, Division below.</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="n"/>
+      <c r="C13" s="8" t="n"/>
+      <c r="D13" s="8" t="n"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>• Plus one Fraction of Amounts and one Percentages of Amounts question, to check the ceiling too.</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="8" t="n"/>
+      <c r="D14" s="8" t="n"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>• Watch: confident or hesitant, mental or written, can she explain the method.</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n"/>
+      <c r="C15" s="8" t="n"/>
+      <c r="D15" s="8" t="n"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>• Then decide: stay on Addition/Subtraction tonight, or move faster into next week's content.</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="n"/>
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="8" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>DAILY PRACTICE (separate from the weekly session below)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>• 10 to 15 min most days: Corbettmaths Primary 5-a-day, not a new topic.</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="n"/>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="10" t="n"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>• Start Silver tier. Move to Gold if too easy after a week or two, Bronze if a struggle.</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="n"/>
+      <c r="C20" s="10" t="n"/>
+      <c r="D20" s="10" t="n"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>• One PDF per month per tier, print monthly not daily. Answers are a separate page, linked below.</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="n"/>
+      <c r="C21" s="10" t="n"/>
+      <c r="D21" s="10" t="n"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>• Plus 2 to 3 min times tables recall, self tested, no worksheet.</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="n"/>
+      <c r="C22" s="10" t="n"/>
+      <c r="D22" s="10" t="n"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>5-a-day home page, always current</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="n"/>
+      <c r="C23" s="10" t="n"/>
+      <c r="D23" s="11" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="6" t="inlineStr">
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>September, Silver, worksheet</t>
         </is>
       </c>
-      <c r="B19" s="7" t="n"/>
-      <c r="C19" s="7" t="n"/>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="B24" s="10" t="n"/>
+      <c r="C24" s="10" t="n"/>
+      <c r="D24" s="11" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="6" t="inlineStr">
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>October, Silver, worksheet</t>
         </is>
       </c>
-      <c r="B20" s="7" t="n"/>
-      <c r="C20" s="7" t="n"/>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="B25" s="10" t="n"/>
+      <c r="C25" s="10" t="n"/>
+      <c r="D25" s="11" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>September answers, all tiers, index page</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="n"/>
-      <c r="C21" s="7" t="n"/>
-      <c r="D21" s="8" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>October answers, all tiers, index page</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="n"/>
-      <c r="C22" s="7" t="n"/>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="26" customHeight="1">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>November onward: the 5-a-day page lists every month by name, click through the same way.</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="n"/>
-      <c r="C23" s="7" t="n"/>
-      <c r="D23" s="7" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>MOCK PAPER, sit Saturday 9 January 2027</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="26" customHeight="1">
+    <row r="26" ht="20" customHeight="1">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>King Edward's does not publish its own specimen paper online. It sends one directly to registered applicants closer to the date, so that is the single most accurate paper there is, ask the school's admissions office for it once registered.</t>
+          <t>September answers, all tiers</t>
         </is>
       </c>
       <c r="B26" s="10" t="n"/>
       <c r="C26" s="10" t="n"/>
-      <c r="D26" s="10" t="n"/>
-    </row>
-    <row r="27" ht="26" customHeight="1">
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>Until it arrives, the closest genuine match is the real Key Stage 2 SATs papers: pure pencil and paper arithmetic (4,532 minus 19, 3 times 391), and word problems with a show your method box, which is the same style as King Edward's own written section. No algebra beyond what the spec lists, no puzzle style stretch questions.</t>
+          <t>October answers, all tiers</t>
         </is>
       </c>
       <c r="B27" s="10" t="n"/>
       <c r="C27" s="10" t="n"/>
-      <c r="D27" s="10" t="n"/>
-    </row>
-    <row r="28" ht="26" customHeight="1">
-      <c r="A28" s="9" t="inlineStr">
-        <is>
-          <t>Sit Paper 1 (Arithmetic, 30 min) in the morning. Sit Paper 2 (Reasoning, 40 min) later that day or the next day, not back to back, 70 minutes of non calculator work in one sitting is a lot for a first full paper.</t>
-        </is>
-      </c>
-      <c r="B28" s="10" t="n"/>
-      <c r="C28" s="10" t="n"/>
-      <c r="D28" s="10" t="n"/>
-    </row>
-    <row r="29" ht="26" customHeight="1">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>No calculator, one sitting per paper, mark from the official scheme the same day.</t>
-        </is>
-      </c>
-      <c r="B29" s="10" t="n"/>
-      <c r="C29" s="10" t="n"/>
-      <c r="D29" s="10" t="n"/>
-    </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="9" t="inlineStr">
-        <is>
-          <t>Paper 1, Arithmetic, 2024</t>
-        </is>
-      </c>
-      <c r="B30" s="10" t="n"/>
-      <c r="C30" s="10" t="n"/>
-      <c r="D30" s="11" t="inlineStr">
+      <c r="D27" s="11" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="9" t="inlineStr">
-        <is>
-          <t>Paper 2, Reasoning, 2024</t>
-        </is>
-      </c>
-      <c r="B31" s="10" t="n"/>
-      <c r="C31" s="10" t="n"/>
-      <c r="D31" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="9" t="inlineStr">
-        <is>
-          <t>Mark schemes, both papers</t>
-        </is>
-      </c>
-      <c r="B32" s="10" t="n"/>
-      <c r="C32" s="10" t="n"/>
-      <c r="D32" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="26" customHeight="1">
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>MOCK PAPER, sit Saturday 9 January 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>• KES sends its own specimen to registered applicants nearer the date. Ask admissions for it, best source there is.</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="n"/>
+      <c r="C30" s="13" t="n"/>
+      <c r="D30" s="13" t="n"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>• Until then: real KS2 SATs papers 2024, level and style verified against the spec.</t>
+        </is>
+      </c>
+      <c r="B31" s="13" t="n"/>
+      <c r="C31" s="13" t="n"/>
+      <c r="D31" s="13" t="n"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>• Sit Paper 1 (Arithmetic, 30 min) morning. Sit Paper 2 (Reasoning, 40 min) separately, same or next day.</t>
+        </is>
+      </c>
+      <c r="B32" s="13" t="n"/>
+      <c r="C32" s="13" t="n"/>
+      <c r="D32" s="13" t="n"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
       <c r="A33" s="12" t="inlineStr">
         <is>
-          <t>Optional second mock, for exam format rather than exact level: Dulwich College publishes real Year 7 entrance specimen papers, one hour, no calculator, with mark schemes. Most of it matches well, but it is an Entrance AND Scholarship paper, so a couple of questions go beyond King Edward's own spec, for example an algebraic age puzzle and a diagram angle counting puzzle. Skip or lightly treat anything that needs setting up an equation, or that is a pure counting puzzle rather than a named topic.</t>
+          <t>• No calculator, mark from the official scheme same day.</t>
         </is>
       </c>
       <c r="B33" s="13" t="n"/>
       <c r="C33" s="13" t="n"/>
       <c r="D33" s="13" t="n"/>
     </row>
-    <row r="34" ht="22" customHeight="1">
+    <row r="34" ht="20" customHeight="1">
       <c r="A34" s="12" t="inlineStr">
         <is>
-          <t>Dulwich College, Specimen Paper A</t>
+          <t>• Optional second paper: Dulwich College Specimen A, 1hr, no calculator. Skip the age equation question and the angle counting puzzle, both go beyond KES's own spec.</t>
         </is>
       </c>
       <c r="B34" s="13" t="n"/>
       <c r="C34" s="13" t="n"/>
-      <c r="D34" s="14" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="22" customHeight="1">
+      <c r="D34" s="13" t="n"/>
+    </row>
+    <row r="35" ht="20" customHeight="1">
       <c r="A35" s="12" t="inlineStr">
         <is>
-          <t>Dulwich College, Specimen Paper A, mark scheme</t>
+          <t>Paper 1, Arithmetic, 2024</t>
         </is>
       </c>
       <c r="B35" s="13" t="n"/>
@@ -967,38 +942,61 @@
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>TWO THINGS STILL TO CHECK</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="26" customHeight="1">
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>Paper 2, Reasoning, 2024</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="n"/>
+      <c r="C36" s="13" t="n"/>
+      <c r="D36" s="14" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>Mark schemes, both papers</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="n"/>
+      <c r="C37" s="13" t="n"/>
+      <c r="D37" s="14" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
       <c r="A38" s="12" t="inlineStr">
         <is>
-          <t>1. Half term is assumed as 27 Oct below. If the school's actual half term is a different week, move that row's date and shift everything after it by the same gap.</t>
+          <t>Dulwich College, Specimen Paper A</t>
         </is>
       </c>
       <c r="B38" s="13" t="n"/>
       <c r="C38" s="13" t="n"/>
-      <c r="D38" s="13" t="n"/>
-      <c r="E38" s="13" t="n"/>
-      <c r="F38" s="13" t="n"/>
-      <c r="G38" s="13" t="n"/>
-    </row>
-    <row r="39" ht="26" customHeight="1">
+      <c r="D38" s="14" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
       <c r="A39" s="12" t="inlineStr">
         <is>
-          <t>2. The 22 Dec and 29 Dec sessions may fall inside the school's Christmas break, not before it. Confirm the actual last day of term. If those two Tuesdays are holiday, either hold both sessions anyway as one off arrangements, or send that fortnight's two packs by message for home practice only and pick the live sessions back up in January.</t>
+          <t>Dulwich College, Specimen Paper A, mark scheme</t>
         </is>
       </c>
       <c r="B39" s="13" t="n"/>
       <c r="C39" s="13" t="n"/>
-      <c r="D39" s="13" t="n"/>
-      <c r="E39" s="13" t="n"/>
-      <c r="F39" s="13" t="n"/>
-      <c r="G39" s="13" t="n"/>
+      <c r="D39" s="14" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="26" customHeight="1">
       <c r="A41" s="15" t="n">
@@ -1029,11 +1027,11 @@
       </c>
       <c r="G41" s="15" t="inlineStr">
         <is>
-          <t>See TODAY block above before starting</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="32" customHeight="1">
+          <t>See TODAY block above first</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
       <c r="A42" s="18" t="n">
         <v>1</v>
       </c>
@@ -1062,11 +1060,11 @@
       </c>
       <c r="G42" s="18" t="inlineStr">
         <is>
-          <t>See TODAY block above before starting</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="32" customHeight="1">
+          <t>See TODAY block above first</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
       <c r="A43" s="21" t="n">
         <v>2</v>
       </c>
@@ -1095,7 +1093,7 @@
       </c>
       <c r="G43" s="21" t="inlineStr"/>
     </row>
-    <row r="44" ht="32" customHeight="1">
+    <row r="44" ht="30" customHeight="1">
       <c r="A44" s="21" t="n">
         <v>2</v>
       </c>
@@ -1124,7 +1122,7 @@
       </c>
       <c r="G44" s="21" t="inlineStr"/>
     </row>
-    <row r="45" ht="32" customHeight="1">
+    <row r="45" ht="30" customHeight="1">
       <c r="A45" s="24" t="n">
         <v>3</v>
       </c>
@@ -1153,7 +1151,7 @@
       </c>
       <c r="G45" s="24" t="inlineStr"/>
     </row>
-    <row r="46" ht="32" customHeight="1">
+    <row r="46" ht="30" customHeight="1">
       <c r="A46" s="24" t="n">
         <v>3</v>
       </c>
@@ -1182,7 +1180,7 @@
       </c>
       <c r="G46" s="24" t="inlineStr"/>
     </row>
-    <row r="47" ht="32" customHeight="1">
+    <row r="47" ht="30" customHeight="1">
       <c r="A47" s="21" t="n">
         <v>4</v>
       </c>
@@ -1211,7 +1209,7 @@
       </c>
       <c r="G47" s="21" t="inlineStr"/>
     </row>
-    <row r="48" ht="32" customHeight="1">
+    <row r="48" ht="30" customHeight="1">
       <c r="A48" s="21" t="n">
         <v>4</v>
       </c>
@@ -1240,65 +1238,73 @@
       </c>
       <c r="G48" s="21" t="inlineStr"/>
     </row>
-    <row r="49" ht="32" customHeight="1">
-      <c r="A49" s="24" t="n">
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" s="27" t="n">
         <v>5</v>
       </c>
-      <c r="B49" s="25" t="n">
+      <c r="B49" s="28" t="n">
         <v>46315</v>
       </c>
-      <c r="C49" s="24" t="inlineStr">
+      <c r="C49" s="27" t="inlineStr">
         <is>
           <t>Number</t>
         </is>
       </c>
-      <c r="D49" s="24" t="inlineStr">
+      <c r="D49" s="27" t="inlineStr">
         <is>
           <t>Prime Numbers</t>
         </is>
       </c>
-      <c r="E49" s="26" t="inlineStr">
-        <is>
-          <t>Worksheet</t>
-        </is>
-      </c>
-      <c r="F49" s="26" t="inlineStr">
-        <is>
-          <t>Answers</t>
-        </is>
-      </c>
-      <c r="G49" s="24" t="inlineStr"/>
-    </row>
-    <row r="50" ht="32" customHeight="1">
-      <c r="A50" s="24" t="n">
+      <c r="E49" s="29" t="inlineStr">
+        <is>
+          <t>Worksheet</t>
+        </is>
+      </c>
+      <c r="F49" s="29" t="inlineStr">
+        <is>
+          <t>Answers</t>
+        </is>
+      </c>
+      <c r="G49" s="27" t="inlineStr">
+        <is>
+          <t>School half term, confirm this session happens</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="27" t="n">
         <v>5</v>
       </c>
-      <c r="B50" s="25" t="n">
+      <c r="B50" s="28" t="n">
         <v>46315</v>
       </c>
-      <c r="C50" s="24" t="inlineStr">
+      <c r="C50" s="27" t="inlineStr">
         <is>
           <t>Number</t>
         </is>
       </c>
-      <c r="D50" s="24" t="inlineStr">
+      <c r="D50" s="27" t="inlineStr">
         <is>
           <t>Square Numbers</t>
         </is>
       </c>
-      <c r="E50" s="26" t="inlineStr">
-        <is>
-          <t>Worksheet</t>
-        </is>
-      </c>
-      <c r="F50" s="26" t="inlineStr">
-        <is>
-          <t>Answers</t>
-        </is>
-      </c>
-      <c r="G50" s="24" t="inlineStr"/>
-    </row>
-    <row r="51" ht="32" customHeight="1">
+      <c r="E50" s="29" t="inlineStr">
+        <is>
+          <t>Worksheet</t>
+        </is>
+      </c>
+      <c r="F50" s="29" t="inlineStr">
+        <is>
+          <t>Answers</t>
+        </is>
+      </c>
+      <c r="G50" s="27" t="inlineStr">
+        <is>
+          <t>School half term, confirm this session happens</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1">
       <c r="A51" s="27" t="n">
         <v>6</v>
       </c>
@@ -1327,11 +1333,11 @@
       </c>
       <c r="G51" s="27" t="inlineStr">
         <is>
-          <t>Half term, assumed date, confirm against the school calendar</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="32" customHeight="1">
+          <t>School half term, confirm this session happens</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="30" customHeight="1">
       <c r="A52" s="27" t="n">
         <v>6</v>
       </c>
@@ -1360,11 +1366,11 @@
       </c>
       <c r="G52" s="27" t="inlineStr">
         <is>
-          <t>Half term, assumed date, confirm against the school calendar. Moved earlier so algebra is not all crammed in near the exam</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="32" customHeight="1">
+          <t>School half term, confirm this session happens</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="30" customHeight="1">
       <c r="A53" s="24" t="n">
         <v>7</v>
       </c>
@@ -1393,7 +1399,7 @@
       </c>
       <c r="G53" s="24" t="inlineStr"/>
     </row>
-    <row r="54" ht="32" customHeight="1">
+    <row r="54" ht="30" customHeight="1">
       <c r="A54" s="24" t="n">
         <v>7</v>
       </c>
@@ -1422,7 +1428,7 @@
       </c>
       <c r="G54" s="24" t="inlineStr"/>
     </row>
-    <row r="55" ht="32" customHeight="1">
+    <row r="55" ht="30" customHeight="1">
       <c r="A55" s="21" t="n">
         <v>8</v>
       </c>
@@ -1449,13 +1455,9 @@
           <t>Answers</t>
         </is>
       </c>
-      <c r="G55" s="21" t="inlineStr">
-        <is>
-          <t>Builds 50, 25, 10, 1 per cent of small numbers, correct level</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="32" customHeight="1">
+      <c r="G55" s="21" t="inlineStr"/>
+    </row>
+    <row r="56" ht="30" customHeight="1">
       <c r="A56" s="21" t="n">
         <v>8</v>
       </c>
@@ -1484,7 +1486,7 @@
       </c>
       <c r="G56" s="21" t="inlineStr"/>
     </row>
-    <row r="57" ht="32" customHeight="1">
+    <row r="57" ht="30" customHeight="1">
       <c r="A57" s="24" t="n">
         <v>9</v>
       </c>
@@ -1511,13 +1513,9 @@
           <t>Answers</t>
         </is>
       </c>
-      <c r="G57" s="24" t="inlineStr">
-        <is>
-          <t>Second and final algebra week, deliberately mid term rather than last</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="32" customHeight="1">
+      <c r="G57" s="24" t="inlineStr"/>
+    </row>
+    <row r="58" ht="30" customHeight="1">
       <c r="A58" s="24" t="n">
         <v>9</v>
       </c>
@@ -1544,13 +1542,9 @@
           <t>Answers</t>
         </is>
       </c>
-      <c r="G58" s="24" t="inlineStr">
-        <is>
-          <t>Divides by 4 then adds 7, answer is 13, exactly the skill needed</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="32" customHeight="1">
+      <c r="G58" s="24" t="inlineStr"/>
+    </row>
+    <row r="59" ht="30" customHeight="1">
       <c r="A59" s="21" t="n">
         <v>10</v>
       </c>
@@ -1579,7 +1573,7 @@
       </c>
       <c r="G59" s="21" t="inlineStr"/>
     </row>
-    <row r="60" ht="32" customHeight="1">
+    <row r="60" ht="30" customHeight="1">
       <c r="A60" s="21" t="n">
         <v>10</v>
       </c>
@@ -1608,7 +1602,7 @@
       </c>
       <c r="G60" s="21" t="inlineStr"/>
     </row>
-    <row r="61" ht="32" customHeight="1">
+    <row r="61" ht="30" customHeight="1">
       <c r="A61" s="24" t="n">
         <v>11</v>
       </c>
@@ -1637,7 +1631,7 @@
       </c>
       <c r="G61" s="24" t="inlineStr"/>
     </row>
-    <row r="62" ht="32" customHeight="1">
+    <row r="62" ht="30" customHeight="1">
       <c r="A62" s="24" t="n">
         <v>11</v>
       </c>
@@ -1666,7 +1660,7 @@
       </c>
       <c r="G62" s="24" t="inlineStr"/>
     </row>
-    <row r="63" ht="32" customHeight="1">
+    <row r="63" ht="30" customHeight="1">
       <c r="A63" s="30" t="n">
         <v>12</v>
       </c>
@@ -1695,11 +1689,11 @@
       </c>
       <c r="G63" s="30" t="inlineStr">
         <is>
-          <t>corbettmaths.com, no Primary page exists for this topic</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="32" customHeight="1">
+          <t>corbettmaths.com, no Primary page for this topic</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="30" customHeight="1">
       <c r="A64" s="21" t="n">
         <v>12</v>
       </c>
@@ -1728,7 +1722,7 @@
       </c>
       <c r="G64" s="21" t="inlineStr"/>
     </row>
-    <row r="65" ht="32" customHeight="1">
+    <row r="65" ht="30" customHeight="1">
       <c r="A65" s="30" t="n">
         <v>13</v>
       </c>
@@ -1757,11 +1751,11 @@
       </c>
       <c r="G65" s="30" t="inlineStr">
         <is>
-          <t>Answers from corbettmaths.com, worksheet from Primary</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="32" customHeight="1">
+          <t>Answers from corbettmaths.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="30" customHeight="1">
       <c r="A66" s="24" t="n">
         <v>13</v>
       </c>
@@ -1790,7 +1784,7 @@
       </c>
       <c r="G66" s="24" t="inlineStr"/>
     </row>
-    <row r="67" ht="32" customHeight="1">
+    <row r="67" ht="30" customHeight="1">
       <c r="A67" s="27" t="n">
         <v>14</v>
       </c>
@@ -1819,11 +1813,11 @@
       </c>
       <c r="G67" s="27" t="inlineStr">
         <is>
-          <t>Check this is not inside the Christmas break, see flag above</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="32" customHeight="1">
+          <t>Christmas holiday, not term time, see calendar block above</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="30" customHeight="1">
       <c r="A68" s="27" t="n">
         <v>14</v>
       </c>
@@ -1852,11 +1846,11 @@
       </c>
       <c r="G68" s="27" t="inlineStr">
         <is>
-          <t>Check this is not inside the Christmas break, see flag above</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="32" customHeight="1">
+          <t>Christmas holiday, not term time, see calendar block above</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="30" customHeight="1">
       <c r="A69" s="27" t="n">
         <v>15</v>
       </c>
@@ -1885,139 +1879,143 @@
       </c>
       <c r="G69" s="27" t="inlineStr">
         <is>
-          <t>Check this is not inside the Christmas break, see flag above</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="32" customHeight="1">
-      <c r="A70" s="30" t="n">
+          <t>Christmas holiday, not term time, see calendar block above</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="30" customHeight="1">
+      <c r="A70" s="27" t="n">
         <v>15</v>
       </c>
-      <c r="B70" s="31" t="n">
+      <c r="B70" s="28" t="n">
         <v>46385</v>
       </c>
-      <c r="C70" s="30" t="inlineStr">
+      <c r="C70" s="27" t="inlineStr">
         <is>
           <t>Handling Data</t>
         </is>
       </c>
-      <c r="D70" s="30" t="inlineStr">
+      <c r="D70" s="27" t="inlineStr">
         <is>
           <t>Median, Mode and Range</t>
         </is>
       </c>
-      <c r="E70" s="32" t="inlineStr">
-        <is>
-          <t>Worksheet</t>
-        </is>
-      </c>
-      <c r="F70" s="32" t="inlineStr">
-        <is>
-          <t>Answers</t>
-        </is>
-      </c>
-      <c r="G70" s="30" t="inlineStr">
-        <is>
-          <t>corbettmaths.com, GCSE labelled, genuinely basic level</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="32" customHeight="1">
-      <c r="A71" s="21" t="n">
+      <c r="E70" s="29" t="inlineStr">
+        <is>
+          <t>Worksheet</t>
+        </is>
+      </c>
+      <c r="F70" s="29" t="inlineStr">
+        <is>
+          <t>Answers</t>
+        </is>
+      </c>
+      <c r="G70" s="27" t="inlineStr">
+        <is>
+          <t>Christmas holiday, not term time. corbettmaths.com, GCSE labelled, genuinely basic level</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="30" customHeight="1">
+      <c r="A71" s="27" t="n">
         <v>16</v>
       </c>
-      <c r="B71" s="22" t="n">
+      <c r="B71" s="28" t="n">
         <v>46392</v>
       </c>
-      <c r="C71" s="21" t="inlineStr">
+      <c r="C71" s="27" t="inlineStr">
         <is>
           <t>Handling Data</t>
         </is>
       </c>
-      <c r="D71" s="21" t="inlineStr">
+      <c r="D71" s="27" t="inlineStr">
         <is>
           <t>Bar Charts</t>
         </is>
       </c>
-      <c r="E71" s="23" t="inlineStr">
-        <is>
-          <t>Worksheet</t>
-        </is>
-      </c>
-      <c r="F71" s="23" t="inlineStr">
-        <is>
-          <t>Answers</t>
-        </is>
-      </c>
-      <c r="G71" s="21" t="inlineStr">
-        <is>
-          <t>Three topics this week, they are quick interpretation skills, not heavy computation</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="32" customHeight="1">
-      <c r="A72" s="21" t="n">
+      <c r="E71" s="29" t="inlineStr">
+        <is>
+          <t>Worksheet</t>
+        </is>
+      </c>
+      <c r="F71" s="29" t="inlineStr">
+        <is>
+          <t>Answers</t>
+        </is>
+      </c>
+      <c r="G71" s="27" t="inlineStr">
+        <is>
+          <t>Christmas holiday, not term time, see calendar block above</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="30" customHeight="1">
+      <c r="A72" s="27" t="n">
         <v>16</v>
       </c>
-      <c r="B72" s="22" t="n">
+      <c r="B72" s="28" t="n">
         <v>46392</v>
       </c>
-      <c r="C72" s="21" t="inlineStr">
+      <c r="C72" s="27" t="inlineStr">
         <is>
           <t>Handling Data</t>
         </is>
       </c>
-      <c r="D72" s="21" t="inlineStr">
+      <c r="D72" s="27" t="inlineStr">
         <is>
           <t>Pie Charts</t>
         </is>
       </c>
-      <c r="E72" s="23" t="inlineStr">
-        <is>
-          <t>Worksheet</t>
-        </is>
-      </c>
-      <c r="F72" s="23" t="inlineStr">
-        <is>
-          <t>Answers</t>
-        </is>
-      </c>
-      <c r="G72" s="21" t="inlineStr"/>
-    </row>
-    <row r="73" ht="32" customHeight="1">
-      <c r="A73" s="21" t="n">
+      <c r="E72" s="29" t="inlineStr">
+        <is>
+          <t>Worksheet</t>
+        </is>
+      </c>
+      <c r="F72" s="29" t="inlineStr">
+        <is>
+          <t>Answers</t>
+        </is>
+      </c>
+      <c r="G72" s="27" t="inlineStr">
+        <is>
+          <t>Christmas holiday, not term time</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="30" customHeight="1">
+      <c r="A73" s="27" t="n">
         <v>16</v>
       </c>
-      <c r="B73" s="22" t="n">
+      <c r="B73" s="28" t="n">
         <v>46392</v>
       </c>
-      <c r="C73" s="21" t="inlineStr">
+      <c r="C73" s="27" t="inlineStr">
         <is>
           <t>Handling Data</t>
         </is>
       </c>
-      <c r="D73" s="21" t="inlineStr">
+      <c r="D73" s="27" t="inlineStr">
         <is>
           <t>Real-life Graphs (Line Graphs)</t>
         </is>
       </c>
-      <c r="E73" s="23" t="inlineStr">
-        <is>
-          <t>Worksheet</t>
-        </is>
-      </c>
-      <c r="F73" s="23" t="inlineStr">
-        <is>
-          <t>Answers</t>
-        </is>
-      </c>
-      <c r="G73" s="21" t="inlineStr">
-        <is>
-          <t>Book sales, temperature, river depth contexts, correct level</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="32" customHeight="1">
+      <c r="E73" s="29" t="inlineStr">
+        <is>
+          <t>Worksheet</t>
+        </is>
+      </c>
+      <c r="F73" s="29" t="inlineStr">
+        <is>
+          <t>Answers</t>
+        </is>
+      </c>
+      <c r="G73" s="27" t="inlineStr">
+        <is>
+          <t>Christmas holiday, not term time</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="30" customHeight="1">
       <c r="A74" s="33" t="inlineStr">
         <is>
           <t>Mock</t>
@@ -2040,11 +2038,11 @@
       <c r="F74" s="35" t="n"/>
       <c r="G74" s="33" t="inlineStr">
         <is>
-          <t>See the Mock Paper block above for links, instructions and the Dulwich alternative</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="32" customHeight="1">
+          <t>See Mock Paper block above</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="30" customHeight="1">
       <c r="A75" s="36" t="n">
         <v>17</v>
       </c>
@@ -2071,112 +2069,113 @@
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A25:C25"/>
     <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A29:D29"/>
-    <mergeCell ref="A38:G38"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="A26:C26"/>
     <mergeCell ref="A13:D13"/>
     <mergeCell ref="A9:D9"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A39:G39"/>
-    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A30:D30"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A10:C10"/>
     <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A31:C31"/>
     <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A30:C30"/>
     <mergeCell ref="A16:D16"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="A21:D21"/>
     <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A32:D32"/>
     <mergeCell ref="A14:D14"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F65" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F66" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F71" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F65" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F66" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F71" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId77"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>